<commit_message>
ops: CVR band finding and the MetaAtomic time split on the hardening task
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VX3eok6oDApR3Yifg7HiSp
</commit_message>
<xml_diff>
--- a/ops/TidsregInfo.xlsx
+++ b/ops/TidsregInfo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\ops\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A66A23B-6C27-44E4-A490-B65B8F512C17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF7AD779-A14D-4E1D-B3CB-39DE2B7C1A49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{8D3CC28D-01B0-4B92-B81A-8912A5232011}"/>
+    <workbookView xWindow="1560" yWindow="1560" windowWidth="28800" windowHeight="15285" xr2:uid="{8D3CC28D-01B0-4B92-B81A-8912A5232011}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="26">
   <si>
     <t>Projektnr</t>
   </si>
@@ -53,18 +53,12 @@
     <t>Tystofte</t>
   </si>
   <si>
-    <t>datakilder</t>
-  </si>
-  <si>
     <t>Finansforbundet</t>
   </si>
   <si>
     <t>4053-01</t>
   </si>
   <si>
-    <t>Møder</t>
-  </si>
-  <si>
     <t>Firma</t>
   </si>
   <si>
@@ -116,16 +110,13 @@
     <t>230-02</t>
   </si>
   <si>
-    <t>?</t>
-  </si>
-  <si>
-    <t>6013-?</t>
-  </si>
-  <si>
     <t>6001-01</t>
   </si>
   <si>
     <t>Vestforbraending</t>
+  </si>
+  <si>
+    <t>4058-1</t>
   </si>
 </sst>
 </file>
@@ -504,20 +495,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97579870-79A3-44CC-9E7B-AAD4BDA85979}">
   <dimension ref="A1:I32"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.33203125" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="20.28515625" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" style="3" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="27.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.6640625" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -529,63 +520,63 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H2" s="1"/>
       <c r="I2" s="2"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
         <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>25</v>
       </c>
       <c r="H3" s="1"/>
       <c r="I3" s="2"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>12</v>
-      </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H4" s="1"/>
       <c r="I4" s="2"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C5" s="3">
         <v>222</v>
@@ -596,168 +587,165 @@
       <c r="H5" s="1"/>
       <c r="I5" s="2"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D6">
         <v>600003</v>
       </c>
       <c r="E6" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H6" s="1"/>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>26</v>
+        <v>15</v>
+      </c>
+      <c r="C7" s="3">
+        <v>6013</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="2"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>25</v>
       </c>
+      <c r="D8">
+        <v>400760</v>
+      </c>
       <c r="H8" s="1"/>
       <c r="I8" s="2"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>5</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" t="s">
-        <v>7</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="2"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
         <v>3</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="2"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H11" s="1"/>
       <c r="I11" s="2"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H12" s="1"/>
       <c r="I12" s="2"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H13" s="1"/>
       <c r="I13" s="2"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H14" s="1"/>
       <c r="I14" s="2"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H15" s="1"/>
       <c r="I15" s="2"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="H16" s="1"/>
       <c r="I16" s="2"/>
     </row>
-    <row r="17" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H17" s="1"/>
       <c r="I17" s="2"/>
     </row>
-    <row r="18" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H18" s="1"/>
       <c r="I18" s="2"/>
     </row>
-    <row r="19" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H19" s="1"/>
       <c r="I19" s="2"/>
     </row>
-    <row r="20" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H20" s="1"/>
       <c r="I20" s="2"/>
     </row>
-    <row r="21" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H21" s="1"/>
       <c r="I21" s="2"/>
     </row>
-    <row r="22" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H22" s="1"/>
       <c r="I22" s="2"/>
     </row>
-    <row r="23" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H23" s="1"/>
       <c r="I23" s="2"/>
     </row>
-    <row r="24" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H24" s="1"/>
       <c r="I24" s="2"/>
     </row>
-    <row r="25" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H25" s="1"/>
       <c r="I25" s="2"/>
     </row>
-    <row r="26" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H26" s="1"/>
       <c r="I26" s="2"/>
     </row>
-    <row r="27" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H27" s="1"/>
       <c r="I27" s="2"/>
     </row>
-    <row r="28" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H28" s="1"/>
       <c r="I28" s="2"/>
     </row>
-    <row r="29" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H29" s="1"/>
       <c r="I29" s="2"/>
     </row>
-    <row r="30" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H30" s="1"/>
       <c r="I30" s="2"/>
     </row>
-    <row r="31" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H31" s="1"/>
       <c r="I31" s="2"/>
     </row>
-    <row r="32" spans="8:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="8:9" x14ac:dyDescent="0.25">
       <c r="H32" s="1"/>
     </row>
   </sheetData>

</xml_diff>